<commit_message>
Updating project to GitHub repo
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -3,19 +3,15 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sonal\eclipse-workspace\Wipro_CapStone_Project\src\test\resources\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{495FC680-3EAB-432A-87C4-DD8DB560137E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{5DA6B01A-89A0-40E8-A90B-E3C854CFB70B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{0F6B139C-D9F3-4CCA-BE57-5528D559D41A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0F6B139C-D9F3-4CCA-BE57-5528D559D41A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -434,6 +430,9 @@
   <cols>
     <col min="2" max="2" width="12.6640625" customWidth="1"/>
     <col min="3" max="3" width="18.5546875" customWidth="1"/>
+    <col min="4" max="4" width="12.21875" customWidth="1"/>
+    <col min="5" max="5" width="14.5546875" customWidth="1"/>
+    <col min="6" max="6" width="11.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>